<commit_message>
Update TEGR Excel spreadsheets to latest versions
</commit_message>
<xml_diff>
--- a/TEGR_10x10_Matrix_WORKING.xlsx
+++ b/TEGR_10x10_Matrix_WORKING.xlsx
@@ -20,10 +20,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.00000"/>
-    <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="0.00000000000"/>
-    <numFmt numFmtId="167" formatCode="0.0E+00"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
+    <numFmt numFmtId="167" formatCode="0.00000000000"/>
+    <numFmt numFmtId="168" formatCode="0.0E+00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -158,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -194,11 +194,55 @@
         <color rgb="00e94560"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00333333"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00333333"/>
+      </right>
+      <top style="thin">
+        <color rgb="00333333"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00333333"/>
+      </right>
+      <top style="thin">
+        <color rgb="00333333"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00333333"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00333333"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00333333"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -230,16 +274,16 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -254,13 +298,13 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,10 +313,33 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -674,6 +741,23 @@
           <t>TEGR 10x10 JACOBIAN MATRIX ENGINE + TICK SIMULATOR</t>
         </is>
       </c>
+      <c r="C1" s="26" t="n"/>
+      <c r="D1" s="26" t="n"/>
+      <c r="E1" s="26" t="n"/>
+      <c r="F1" s="26" t="n"/>
+      <c r="G1" s="26" t="n"/>
+      <c r="H1" s="26" t="n"/>
+      <c r="I1" s="26" t="n"/>
+      <c r="J1" s="26" t="n"/>
+      <c r="K1" s="26" t="n"/>
+      <c r="L1" s="26" t="n"/>
+      <c r="M1" s="26" t="n"/>
+      <c r="N1" s="26" t="n"/>
+      <c r="O1" s="26" t="n"/>
+      <c r="P1" s="26" t="n"/>
+      <c r="Q1" s="26" t="n"/>
+      <c r="R1" s="26" t="n"/>
+      <c r="S1" s="27" t="n"/>
       <c r="T1" s="1" t="n"/>
       <c r="U1" s="1" t="n"/>
       <c r="V1" s="1" t="n"/>
@@ -686,6 +770,23 @@
           <t>GOLD cells = type your numbers  |  GREEN cells = auto-computed  |  ORANGE = tick output</t>
         </is>
       </c>
+      <c r="C2" s="26" t="n"/>
+      <c r="D2" s="26" t="n"/>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+      <c r="J2" s="26" t="n"/>
+      <c r="K2" s="26" t="n"/>
+      <c r="L2" s="26" t="n"/>
+      <c r="M2" s="26" t="n"/>
+      <c r="N2" s="26" t="n"/>
+      <c r="O2" s="26" t="n"/>
+      <c r="P2" s="26" t="n"/>
+      <c r="Q2" s="26" t="n"/>
+      <c r="R2" s="26" t="n"/>
+      <c r="S2" s="27" t="n"/>
       <c r="T2" s="1" t="n"/>
       <c r="U2" s="1" t="n"/>
       <c r="V2" s="1" t="n"/>
@@ -706,6 +807,15 @@
           <t>10x10 JACOBIAN J (for stability analysis / PySINDy)</t>
         </is>
       </c>
+      <c r="K3" s="26" t="n"/>
+      <c r="L3" s="26" t="n"/>
+      <c r="M3" s="26" t="n"/>
+      <c r="N3" s="26" t="n"/>
+      <c r="O3" s="26" t="n"/>
+      <c r="P3" s="26" t="n"/>
+      <c r="Q3" s="26" t="n"/>
+      <c r="R3" s="26" t="n"/>
+      <c r="S3" s="27" t="n"/>
       <c r="T3" s="1" t="n"/>
       <c r="U3" s="1" t="n"/>
       <c r="V3" s="1" t="n"/>
@@ -718,6 +828,7 @@
           <t>STATE VECTOR X (INPUT)</t>
         </is>
       </c>
+      <c r="C4" s="27" t="n"/>
       <c r="D4" s="1" t="n"/>
       <c r="E4" s="1" t="n"/>
       <c r="F4" s="5" t="inlineStr">
@@ -725,6 +836,7 @@
           <t>HELPERS (auto)</t>
         </is>
       </c>
+      <c r="G4" s="27" t="n"/>
       <c r="H4" s="1" t="n"/>
       <c r="I4" s="1" t="n"/>
       <c r="J4" s="6" t="inlineStr">
@@ -844,7 +956,7 @@
       <c r="R5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S5" s="11" t="n">
+      <c r="S5" s="28" t="n">
         <v>1</v>
       </c>
       <c r="T5" s="1" t="n"/>
@@ -899,7 +1011,7 @@
       <c r="M6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="29">
         <f>1/(C14*C12)</f>
         <v/>
       </c>
@@ -909,14 +1021,14 @@
       <c r="P6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="Q6" s="12">
+      <c r="Q6" s="29">
         <f>-C9/(C14*C12^2)</f>
         <v/>
       </c>
       <c r="R6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S6" s="12">
+      <c r="S6" s="29">
         <f>-C9/(C14^2*C12)</f>
         <v/>
       </c>
@@ -975,21 +1087,21 @@
       <c r="N7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="O7" s="12">
+      <c r="O7" s="29">
         <f>1/(C14*C12)</f>
         <v/>
       </c>
       <c r="P7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" s="12">
+      <c r="Q7" s="29">
         <f>-C10/(C14*C12^2)</f>
         <v/>
       </c>
       <c r="R7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S7" s="12">
+      <c r="S7" s="29">
         <f>-C10/(C14^2*C12)</f>
         <v/>
       </c>
@@ -1051,18 +1163,18 @@
       <c r="O8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="29">
         <f>1/(C14*C12)</f>
         <v/>
       </c>
-      <c r="Q8" s="12">
+      <c r="Q8" s="29">
         <f>-C11/(C14*C12^2)</f>
         <v/>
       </c>
       <c r="R8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S8" s="12">
+      <c r="S8" s="29">
         <f>-C11/(C14^2*C12)</f>
         <v/>
       </c>
@@ -1109,37 +1221,37 @@
       <c r="J9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="29">
         <f>C18*C12*(3*C6^2-(C6^2+C7^2+C8^2))/G5^5</f>
         <v/>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="29">
         <f>C18*C12*3*C6*C7/G5^5</f>
         <v/>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="29">
         <f>C18*C12*3*C6*C8/G5^5</f>
         <v/>
       </c>
       <c r="N9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="O9" s="12">
+      <c r="O9" s="29">
         <f>(C19*C24+C20*C27)/(C14*C12)</f>
         <v/>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="29">
         <f>-(C19*C23+C20*C26)/(C14*C12)</f>
         <v/>
       </c>
-      <c r="Q9" s="12">
-        <f>-C18*C6/G12</f>
+      <c r="Q9" s="29">
+        <f>-C18*C6/G12-(G22+G26)/C12</f>
         <v/>
       </c>
       <c r="R9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S9" s="12">
+      <c r="S9" s="29">
         <f>-((C19*C24+C20*C27)*C10-(C19*C23+C20*C26)*C11)/(C14^2*C12)</f>
         <v/>
       </c>
@@ -1186,37 +1298,37 @@
       <c r="J10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="29">
         <f>C18*C12*3*C7*C6/G5^5</f>
         <v/>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="29">
         <f>C18*C12*(3*C7^2-(C6^2+C7^2+C8^2))/G5^5</f>
         <v/>
       </c>
-      <c r="M10" s="12">
+      <c r="M10" s="29">
         <f>C18*C12*3*C7*C8/G5^5</f>
         <v/>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="29">
         <f>-(C19*C24+C20*C27)/(C14*C12)</f>
         <v/>
       </c>
       <c r="O10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="P10" s="12">
+      <c r="P10" s="29">
         <f>(C19*C22+C20*C25)/(C14*C12)</f>
         <v/>
       </c>
-      <c r="Q10" s="12">
-        <f>-C18*C7/G12</f>
+      <c r="Q10" s="29">
+        <f>-C18*C7/G12-(G23+G27)/C12</f>
         <v/>
       </c>
       <c r="R10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="12">
+      <c r="S10" s="29">
         <f>((C19*C24+C20*C27)*C9-(C19*C22+C20*C25)*C11)/(C14^2*C12)</f>
         <v/>
       </c>
@@ -1263,37 +1375,37 @@
       <c r="J11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="29">
         <f>C18*C12*3*C8*C6/G5^5</f>
         <v/>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="29">
         <f>C18*C12*3*C8*C7/G5^5</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="29">
         <f>C18*C12*(3*C8^2-(C6^2+C7^2+C8^2))/G5^5</f>
         <v/>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="29">
         <f>(C19*C23+C20*C26)/(C14*C12)</f>
         <v/>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="29">
         <f>-(C19*C22+C20*C25)/(C14*C12)</f>
         <v/>
       </c>
       <c r="P11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="Q11" s="12">
-        <f>-C18*C8/G12</f>
+      <c r="Q11" s="29">
+        <f>-C18*C8/G12-(G24+G28)/C12</f>
         <v/>
       </c>
       <c r="R11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S11" s="12">
+      <c r="S11" s="29">
         <f>-((C19*C23+C20*C26)*C9-(C19*C22+C20*C25)*C10)/(C14^2*C12)</f>
         <v/>
       </c>
@@ -1417,14 +1529,14 @@
       <c r="P13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="Q13" s="12">
+      <c r="Q13" s="29">
         <f>C14*C28^2/C29</f>
         <v/>
       </c>
       <c r="R13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="S13" s="12">
+      <c r="S13" s="29">
         <f>C12*C28^2/C29</f>
         <v/>
       </c>
@@ -1469,16 +1581,16 @@
       <c r="M14" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="12">
-        <f>C14^2*(-C18*C12*C6/G12)/(C12^2*C28^2*C14)</f>
-        <v/>
-      </c>
-      <c r="O14" s="12">
-        <f>C14^2*(-C18*C12*C7/G12)/(C12^2*C28^2*C14)</f>
-        <v/>
-      </c>
-      <c r="P14" s="12">
-        <f>C14^2*(-C18*C12*C8/G12)/(C12^2*C28^2*C14)</f>
+      <c r="N14" s="29">
+        <f>G30/(C14*C12^2*C28^2)-(C9*G30+C10*G31+C11*G32)*C9/(C14^3*C12^4*C28^4)</f>
+        <v/>
+      </c>
+      <c r="O14" s="29">
+        <f>G31/(C14*C12^2*C28^2)-(C9*G30+C10*G31+C11*G32)*C10/(C14^3*C12^4*C28^4)</f>
+        <v/>
+      </c>
+      <c r="P14" s="29">
+        <f>G32/(C14*C12^2*C28^2)-(C9*G30+C10*G31+C11*G32)*C11/(C14^3*C12^4*C28^4)</f>
         <v/>
       </c>
       <c r="Q14" s="10" t="n">
@@ -1552,6 +1664,7 @@
           <t>PARAMETERS (INPUT)</t>
         </is>
       </c>
+      <c r="C17" s="27" t="n"/>
       <c r="D17" s="1" t="n"/>
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="5" t="inlineStr">
@@ -1559,6 +1672,7 @@
           <t>FORCES (auto)</t>
         </is>
       </c>
+      <c r="G17" s="27" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
       <c r="J17" s="1" t="n"/>
@@ -2252,6 +2366,8 @@
           <t>f(X) DIRECT EQUATIONS OF MOTION</t>
         </is>
       </c>
+      <c r="G35" s="26" t="n"/>
+      <c r="H35" s="27" t="n"/>
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="n"/>
       <c r="K35" s="1" t="n"/>
@@ -2316,7 +2432,7 @@
           <t>dt/dt</t>
         </is>
       </c>
-      <c r="G37" s="14">
+      <c r="G37" s="30">
         <f>C14</f>
         <v/>
       </c>
@@ -2352,7 +2468,7 @@
           <t>dx/dt</t>
         </is>
       </c>
-      <c r="G38" s="14">
+      <c r="G38" s="30">
         <f>G8</f>
         <v/>
       </c>
@@ -2388,7 +2504,7 @@
           <t>dy/dt</t>
         </is>
       </c>
-      <c r="G39" s="14">
+      <c r="G39" s="30">
         <f>G9</f>
         <v/>
       </c>
@@ -2424,7 +2540,7 @@
           <t>dz/dt</t>
         </is>
       </c>
-      <c r="G40" s="14">
+      <c r="G40" s="30">
         <f>G10</f>
         <v/>
       </c>
@@ -2460,7 +2576,7 @@
           <t>dpx/dt</t>
         </is>
       </c>
-      <c r="G41" s="14">
+      <c r="G41" s="30">
         <f>G30</f>
         <v/>
       </c>
@@ -2496,7 +2612,7 @@
           <t>dpy/dt</t>
         </is>
       </c>
-      <c r="G42" s="14">
+      <c r="G42" s="30">
         <f>G31</f>
         <v/>
       </c>
@@ -2532,7 +2648,7 @@
           <t>dpz/dt</t>
         </is>
       </c>
-      <c r="G43" s="14">
+      <c r="G43" s="30">
         <f>G32</f>
         <v/>
       </c>
@@ -2568,7 +2684,7 @@
           <t>dm0/dt</t>
         </is>
       </c>
-      <c r="G44" s="14" t="n">
+      <c r="G44" s="30" t="n">
         <v>0</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2603,7 +2719,7 @@
           <t>dth/dt</t>
         </is>
       </c>
-      <c r="G45" s="14">
+      <c r="G45" s="30">
         <f>C14*C12*C28^2/C29</f>
         <v/>
       </c>
@@ -2639,7 +2755,7 @@
           <t>dgam/dt</t>
         </is>
       </c>
-      <c r="G46" s="14" t="inlineStr">
+      <c r="G46" s="30" t="inlineStr">
         <is>
           <t>computed in sync</t>
         </is>
@@ -2722,6 +2838,12 @@
           <t>THE TICK ENGINE  --  Section 4 Momentum-Velocity Sync</t>
         </is>
       </c>
+      <c r="C49" s="26" t="n"/>
+      <c r="D49" s="26" t="n"/>
+      <c r="E49" s="26" t="n"/>
+      <c r="F49" s="26" t="n"/>
+      <c r="G49" s="26" t="n"/>
+      <c r="H49" s="27" t="n"/>
       <c r="I49" s="1" t="n"/>
       <c r="J49" s="1" t="n"/>
       <c r="K49" s="1" t="n"/>
@@ -2745,6 +2867,12 @@
           <t>Each step computes X(t+dt) from X(t). Copy RESULT back to inputs to advance.</t>
         </is>
       </c>
+      <c r="C50" s="26" t="n"/>
+      <c r="D50" s="26" t="n"/>
+      <c r="E50" s="26" t="n"/>
+      <c r="F50" s="26" t="n"/>
+      <c r="G50" s="26" t="n"/>
+      <c r="H50" s="27" t="n"/>
       <c r="I50" s="1" t="n"/>
       <c r="J50" s="1" t="n"/>
       <c r="K50" s="1" t="n"/>
@@ -2809,6 +2937,8 @@
           <t>CONSERVATION CHECKS</t>
         </is>
       </c>
+      <c r="G52" s="26" t="n"/>
+      <c r="H52" s="27" t="n"/>
       <c r="I52" s="1" t="n"/>
       <c r="J52" s="1" t="n"/>
       <c r="K52" s="1" t="n"/>
@@ -2832,7 +2962,7 @@
           <t>px_temp</t>
         </is>
       </c>
-      <c r="C53" s="19">
+      <c r="C53" s="31">
         <f>C9+G30*C30</f>
         <v/>
       </c>
@@ -2847,7 +2977,7 @@
           <t>m_inv BEFORE</t>
         </is>
       </c>
-      <c r="G53" s="20">
+      <c r="G53" s="32">
         <f>SQRT((C14*C12)^2-(C9^2+C10^2+C11^2))</f>
         <v/>
       </c>
@@ -2879,7 +3009,7 @@
           <t>py_temp</t>
         </is>
       </c>
-      <c r="C54" s="19">
+      <c r="C54" s="31">
         <f>C10+G31*C30</f>
         <v/>
       </c>
@@ -2890,13 +3020,13 @@
           <t>m_inv AFTER</t>
         </is>
       </c>
-      <c r="G54" s="20">
-        <f>SQRT((C75*C91)^2-(C78^2+C79^2+C80^2))</f>
+      <c r="G54" s="32">
+        <f>SQRT((C14*C12+(G30*C69+G31*C70+G32*C71)*C30/C28^2)^2-C56^2)</f>
         <v/>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>should match BEFORE</t>
+          <t>Euler-step invariant mass (genuine check)</t>
         </is>
       </c>
       <c r="I54" s="1" t="n"/>
@@ -2922,7 +3052,7 @@
           <t>pz_temp</t>
         </is>
       </c>
-      <c r="C55" s="19">
+      <c r="C55" s="31">
         <f>C11+G32*C30</f>
         <v/>
       </c>
@@ -2933,7 +3063,7 @@
           <t>MASS LEAKAGE</t>
         </is>
       </c>
-      <c r="G55" s="21">
+      <c r="G55" s="33">
         <f>ABS(G53-G54)</f>
         <v/>
       </c>
@@ -2965,7 +3095,7 @@
           <t>|p_temp|</t>
         </is>
       </c>
-      <c r="C56" s="19">
+      <c r="C56" s="31">
         <f>SQRT(C53^2+C54^2+C55^2)</f>
         <v/>
       </c>
@@ -3077,8 +3207,8 @@
           <t>denom</t>
         </is>
       </c>
-      <c r="C59" s="19">
-        <f>SQRT(C12^2+C56^2)</f>
+      <c r="C59" s="31">
+        <f>SQRT((C12*C28)^2+C56^2)/C28</f>
         <v/>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -3113,7 +3243,7 @@
           <t>vx_temp</t>
         </is>
       </c>
-      <c r="C60" s="19">
+      <c r="C60" s="31">
         <f>C53/C59</f>
         <v/>
       </c>
@@ -3152,7 +3282,7 @@
           <t>vy_temp</t>
         </is>
       </c>
-      <c r="C61" s="19">
+      <c r="C61" s="31">
         <f>C54/C59</f>
         <v/>
       </c>
@@ -3191,7 +3321,7 @@
           <t>vz_temp</t>
         </is>
       </c>
-      <c r="C62" s="19">
+      <c r="C62" s="31">
         <f>C55/C59</f>
         <v/>
       </c>
@@ -3230,7 +3360,7 @@
           <t>|v_temp|</t>
         </is>
       </c>
-      <c r="C63" s="19">
+      <c r="C63" s="31">
         <f>SQRT(C60^2+C61^2+C62^2)</f>
         <v/>
       </c>
@@ -3324,7 +3454,7 @@
           <t>cap_val</t>
         </is>
       </c>
-      <c r="C66" s="19">
+      <c r="C66" s="31">
         <f>C31*C28</f>
         <v/>
       </c>
@@ -3392,7 +3522,7 @@
           <t>scale</t>
         </is>
       </c>
-      <c r="C68" s="19">
+      <c r="C68" s="31">
         <f>IF(C63&gt;=C66,C66/C63,1)</f>
         <v/>
       </c>
@@ -3428,7 +3558,7 @@
           <t>vx_cap</t>
         </is>
       </c>
-      <c r="C69" s="19">
+      <c r="C69" s="31">
         <f>C60*C68</f>
         <v/>
       </c>
@@ -3460,7 +3590,7 @@
           <t>vy_cap</t>
         </is>
       </c>
-      <c r="C70" s="19">
+      <c r="C70" s="31">
         <f>C61*C68</f>
         <v/>
       </c>
@@ -3492,7 +3622,7 @@
           <t>vz_cap</t>
         </is>
       </c>
-      <c r="C71" s="19">
+      <c r="C71" s="31">
         <f>C62*C68</f>
         <v/>
       </c>
@@ -3524,7 +3654,7 @@
           <t>|v_cap|</t>
         </is>
       </c>
-      <c r="C72" s="19">
+      <c r="C72" s="31">
         <f>SQRT(C69^2+C70^2+C71^2)</f>
         <v/>
       </c>
@@ -3618,7 +3748,7 @@
           <t>gamma_new</t>
         </is>
       </c>
-      <c r="C75" s="19">
+      <c r="C75" s="31">
         <f>1/SQRT(1-C72^2/C28^2)</f>
         <v/>
       </c>
@@ -3712,7 +3842,7 @@
           <t>px_new</t>
         </is>
       </c>
-      <c r="C78" s="19">
+      <c r="C78" s="31">
         <f>C75*C12*C69</f>
         <v/>
       </c>
@@ -3744,7 +3874,7 @@
           <t>py_new</t>
         </is>
       </c>
-      <c r="C79" s="19">
+      <c r="C79" s="31">
         <f>C75*C12*C70</f>
         <v/>
       </c>
@@ -3775,7 +3905,7 @@
           <t>pz_new</t>
         </is>
       </c>
-      <c r="C80" s="19">
+      <c r="C80" s="31">
         <f>C75*C12*C71</f>
         <v/>
       </c>
@@ -3786,6 +3916,8 @@
           <t>RESULT: X(t + dt)  --  Copy these back to C5:C14</t>
         </is>
       </c>
+      <c r="C83" s="26" t="n"/>
+      <c r="D83" s="27" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="7" t="inlineStr">
@@ -3793,7 +3925,7 @@
           <t>t_new</t>
         </is>
       </c>
-      <c r="C84" s="24">
+      <c r="C84" s="34">
         <f>C5+C30</f>
         <v/>
       </c>
@@ -3809,7 +3941,7 @@
           <t>x_new</t>
         </is>
       </c>
-      <c r="C85" s="24">
+      <c r="C85" s="34">
         <f>C6+C69*C30</f>
         <v/>
       </c>
@@ -3825,7 +3957,7 @@
           <t>y_new</t>
         </is>
       </c>
-      <c r="C86" s="24">
+      <c r="C86" s="34">
         <f>C7+C70*C30</f>
         <v/>
       </c>
@@ -3841,7 +3973,7 @@
           <t>z_new</t>
         </is>
       </c>
-      <c r="C87" s="24">
+      <c r="C87" s="34">
         <f>C8+C71*C30</f>
         <v/>
       </c>
@@ -3857,7 +3989,7 @@
           <t>px_new</t>
         </is>
       </c>
-      <c r="C88" s="24">
+      <c r="C88" s="34">
         <f>C78</f>
         <v/>
       </c>
@@ -3873,7 +4005,7 @@
           <t>py_new</t>
         </is>
       </c>
-      <c r="C89" s="24">
+      <c r="C89" s="34">
         <f>C79</f>
         <v/>
       </c>
@@ -3889,7 +4021,7 @@
           <t>pz_new</t>
         </is>
       </c>
-      <c r="C90" s="24">
+      <c r="C90" s="34">
         <f>C80</f>
         <v/>
       </c>
@@ -3905,7 +4037,7 @@
           <t>m0_new</t>
         </is>
       </c>
-      <c r="C91" s="24">
+      <c r="C91" s="34">
         <f>C12</f>
         <v/>
       </c>
@@ -3921,7 +4053,7 @@
           <t>theta_new</t>
         </is>
       </c>
-      <c r="C92" s="24">
+      <c r="C92" s="34">
         <f>MOD(C13+C75*C12*C28^2/C29*C30, 2*PI())</f>
         <v/>
       </c>
@@ -3937,7 +4069,7 @@
           <t>gamma_new</t>
         </is>
       </c>
-      <c r="C93" s="24">
+      <c r="C93" s="34">
         <f>C75</f>
         <v/>
       </c>
@@ -3990,7 +4122,6 @@
     </row>
     <row r="2">
       <c r="A2" s="25" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -4014,7 +4145,6 @@
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="25" t="inlineStr">
@@ -4038,7 +4168,6 @@
     </row>
     <row r="8">
       <c r="A8" s="25" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
@@ -4094,7 +4223,6 @@
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
@@ -4118,7 +4246,6 @@
     </row>
     <row r="18">
       <c r="A18" s="25" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
@@ -4158,7 +4285,6 @@
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
@@ -4198,7 +4324,6 @@
     </row>
     <row r="28">
       <c r="A28" s="25" t="inlineStr"/>
-      <c r="B28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="25" t="inlineStr"/>
@@ -4242,7 +4367,6 @@
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr"/>
-      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="25" t="inlineStr"/>
@@ -4302,8 +4426,6 @@
           <t>ENTANGLEMENT ADJACENCY TENSOR Wij</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4311,14 +4433,8 @@
           <t>(Paper 2: ER=EPR and AMPS Firewall)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4375,19 +4491,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>COMPUTED</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4399,7 +4509,6 @@
         <f>ABS(B5-C5)</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4432,11 +4541,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -4447,21 +4552,14 @@
         <f>IF(B10&lt;B11,"ACTIVE (wormhole open)","SNAPPED -&gt; FIREWALL")</f>
         <v/>
       </c>
-      <c r="C14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>IF SNAPPED:</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">

</xml_diff>

<commit_message>
Fix time dilation inversion in TEGR Matrix spreadsheet (4 cells: C92, G45, Q13, S13)
The phase clock was multiplying by gamma instead of dividing by gamma,
causing the internal frequency to spike at relativistic speeds instead
of dilating. This is the exact same Einstein Stick bug that was fixed
in the Python engine.

Fixes:
- C92: Tick Engine phase update (m0/gamma, not gamma*m0)
- G45: Direct EOM theta_dot (m0/gamma, not gamma*m0)
- Q13: Jacobian d(theta_dot)/dm0 (c^2/(gamma*hbar), not gamma*c^2/hbar)
- S13: Jacobian d(theta_dot)/dgamma (-m0*c^2/(gamma^2*hbar) via power rule)

Backup of original saved as TEGR_10x10_Matrix_WORKING_BACKUP_PRE_PHASE_FIX.xlsx
</commit_message>
<xml_diff>
--- a/TEGR_10x10_Matrix_WORKING.xlsx
+++ b/TEGR_10x10_Matrix_WORKING.xlsx
@@ -1530,14 +1530,14 @@
         <v>0</v>
       </c>
       <c r="Q13" s="29">
-        <f>C14*C28^2/C29</f>
+        <f>C28^2/(C14*C29)</f>
         <v/>
       </c>
       <c r="R13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="S13" s="29">
-        <f>C12*C28^2/C29</f>
+        <f>-C12*C28^2/(C14^2*C29)</f>
         <v/>
       </c>
       <c r="T13" s="1" t="n"/>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="G45" s="30">
-        <f>C14*C12*C28^2/C29</f>
+        <f>(C12/C14)*C28^2/C29</f>
         <v/>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C92" s="34">
-        <f>MOD(C13+C75*C12*C28^2/C29*C30, 2*PI())</f>
+        <f>MOD(C13+(C12/C75)*C28^2/C29*C30, 2*PI())</f>
         <v/>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -4105,7 +4105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:S92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4400,6 +4400,8 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="92"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4412,7 +4414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:S92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4434,7 +4436,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -4491,7 +4492,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -4553,7 +4553,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -4609,6 +4608,8 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="92"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>